<commit_message>
Put a real example in the sample sheet, and find the schedule tab
The download called a sample sheet carried headers and nothing else, so a
planner who opened it, saved it and uploaded it straight back got "no rooms
could be read". It now ships three example rows, two of which share a Room Name
to demonstrate the multi-function grouping the upload is built around.

The parser also took the leftmost sheet, while the workbook has pivot, virtual
schedule and room tabs beside the schedule. It now reads the first sheet that
carries room and function columns, falling back to the old behaviour so an
unrecognised file still reports what it reported before.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/files/RFPilot schedule-example-sheet.xlsx
+++ b/public/files/RFPilot schedule-example-sheet.xlsx
@@ -326,6 +326,120 @@
         <x:v>Special requirements</x:v>
       </x:c>
     </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="0" t="str">
+        <x:v>2027-03-10</x:v>
+      </x:c>
+      <x:c r="B2" s="0" t="str">
+        <x:v>Wednesday</x:v>
+      </x:c>
+      <x:c r="C2" s="0" t="str">
+        <x:v>9:00 AM</x:v>
+      </x:c>
+      <x:c r="D2" s="0" t="str">
+        <x:v>11:30 AM</x:v>
+      </x:c>
+      <x:c r="E2" s="0" t="str">
+        <x:v>Opening Keynote</x:v>
+      </x:c>
+      <x:c r="F2" s="0" t="str">
+        <x:v>Grand Ballroom</x:v>
+      </x:c>
+      <x:c r="G2" s="0" t="str">
+        <x:v>Theater</x:v>
+      </x:c>
+      <x:c r="H2" s="0" t="str">
+        <x:v>450</x:v>
+      </x:c>
+      <x:c r="I2" s="0" t="str">
+        <x:v>CEO</x:v>
+      </x:c>
+      <x:c r="J2" s="0" t="str">
+        <x:v>Alex</x:v>
+      </x:c>
+      <x:c r="K2" s="0" t="str">
+        <x:v>All</x:v>
+      </x:c>
+      <x:c r="L2" s="0" t="str">
+        <x:v>Record keynote</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="0" t="str">
+        <x:v>2027-03-12</x:v>
+      </x:c>
+      <x:c r="B3" s="0" t="str">
+        <x:v>Friday</x:v>
+      </x:c>
+      <x:c r="C3" s="0" t="str">
+        <x:v>3:00 PM</x:v>
+      </x:c>
+      <x:c r="D3" s="0" t="str">
+        <x:v>5:00 PM</x:v>
+      </x:c>
+      <x:c r="E3" s="0" t="str">
+        <x:v>Closing General Session</x:v>
+      </x:c>
+      <x:c r="F3" s="0" t="str">
+        <x:v>Grand Ballroom</x:v>
+      </x:c>
+      <x:c r="G3" s="0" t="str">
+        <x:v>Theater</x:v>
+      </x:c>
+      <x:c r="H3" s="0" t="str">
+        <x:v>430</x:v>
+      </x:c>
+      <x:c r="I3" s="0" t="str">
+        <x:v>CRO</x:v>
+      </x:c>
+      <x:c r="J3" s="0" t="str">
+        <x:v>Alex</x:v>
+      </x:c>
+      <x:c r="K3" s="0" t="str">
+        <x:v>All</x:v>
+      </x:c>
+      <x:c r="L3" s="0" t="str">
+        <x:v>Same room as the keynote</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="0" t="str">
+        <x:v>2027-03-11</x:v>
+      </x:c>
+      <x:c r="B4" s="0" t="str">
+        <x:v>Thursday</x:v>
+      </x:c>
+      <x:c r="C4" s="0" t="str">
+        <x:v>9:00 AM</x:v>
+      </x:c>
+      <x:c r="D4" s="0" t="str">
+        <x:v>12:00 PM</x:v>
+      </x:c>
+      <x:c r="E4" s="0" t="str">
+        <x:v>Breakout A</x:v>
+      </x:c>
+      <x:c r="F4" s="0" t="str">
+        <x:v>Salon 1</x:v>
+      </x:c>
+      <x:c r="G4" s="0" t="str">
+        <x:v>Classroom</x:v>
+      </x:c>
+      <x:c r="H4" s="0" t="str">
+        <x:v>80</x:v>
+      </x:c>
+      <x:c r="I4" s="0" t="str">
+        <x:v>VP Sales</x:v>
+      </x:c>
+      <x:c r="J4" s="0" t="str">
+        <x:v>Jamie</x:v>
+      </x:c>
+      <x:c r="K4" s="0" t="str">
+        <x:v>Advanced</x:v>
+      </x:c>
+      <x:c r="L4" s="0" t="str">
+        <x:v/>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>